<commit_message>
Fix generic table placeholder classification
</commit_message>
<xml_diff>
--- a/benchmarking_automation/output/classified_inventory.xlsx
+++ b/benchmarking_automation/output/classified_inventory.xlsx
@@ -2549,18 +2549,22 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>keyvalue</t>
+          <t>table</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>INLINE_CONTEXT_PRESENT</t>
-        </is>
-      </c>
-      <c r="F65" t="inlineStr"/>
+          <t>TABLE_SYNTAX_MATCH</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>TABLE_SYNTAX_RULE</t>
+        </is>
+      </c>
       <c r="G65" t="inlineStr">
         <is>
           <t>paragraph</t>

</xml_diff>